<commit_message>
Completed Data Driven with Excel.
</commit_message>
<xml_diff>
--- a/ParabankAutomation/src/test/resources/TestData.xlsx
+++ b/ParabankAutomation/src/test/resources/TestData.xlsx
@@ -2,21 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView activeTab="0"/>
-  </bookViews>
   <sheets>
     <sheet state="visible" name="Registration" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="NegativeTestData" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="AccountData" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="LoginData" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="BillPay" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="NegativeTestData" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="AccountData" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="LoginData" sheetId="5" r:id="rId9"/>
   </sheets>
+  <definedNames/>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
   <si>
     <t>First Name</t>
   </si>
@@ -66,12 +65,45 @@
     <t>123-45-6789</t>
   </si>
   <si>
-    <t>Demo_Shubh</t>
+    <t>DemoUser</t>
   </si>
   <si>
     <t>Test@1234</t>
   </si>
   <si>
+    <t>Payee Name</t>
+  </si>
+  <si>
+    <t>Payee address</t>
+  </si>
+  <si>
+    <t>Payee city</t>
+  </si>
+  <si>
+    <t>Payee State</t>
+  </si>
+  <si>
+    <t>Payee zip</t>
+  </si>
+  <si>
+    <t>Payee Phone</t>
+  </si>
+  <si>
+    <t>Payee Amount</t>
+  </si>
+  <si>
+    <t>Shubhank</t>
+  </si>
+  <si>
+    <t>HL 333, Metro Road</t>
+  </si>
+  <si>
+    <t>LDH</t>
+  </si>
+  <si>
+    <t>Punjab</t>
+  </si>
+  <si>
     <t>username</t>
   </si>
   <si>
@@ -85,319 +117,12 @@
   </si>
   <si>
     <t>Hey</t>
-  </si>
-  <si>
-    <t>Shubhs</t>
-  </si>
-  <si>
-    <t>demo</t>
-  </si>
-  <si>
-    <t>bugad1780938465219</t>
-  </si>
-  <si>
-    <t>bugad1780938469409</t>
-  </si>
-  <si>
-    <t>bugad1780938473840</t>
-  </si>
-  <si>
-    <t>bugad1780938477254</t>
-  </si>
-  <si>
-    <t>bugad1780938496120</t>
-  </si>
-  <si>
-    <t>demo1780942368557</t>
-  </si>
-  <si>
-    <t>14343</t>
-  </si>
-  <si>
-    <t>CHECKING</t>
-  </si>
-  <si>
-    <t>demo1780942457104</t>
-  </si>
-  <si>
-    <t>14565</t>
-  </si>
-  <si>
-    <t>14676</t>
-  </si>
-  <si>
-    <t>SAVINGS</t>
-  </si>
-  <si>
-    <t>demo1780942515333</t>
-  </si>
-  <si>
-    <t>demo1780942760400</t>
-  </si>
-  <si>
-    <t>demo1780943121029</t>
-  </si>
-  <si>
-    <t>demo1780943233862</t>
-  </si>
-  <si>
-    <t>demo1780943608757</t>
-  </si>
-  <si>
-    <t>demo1780943648312</t>
-  </si>
-  <si>
-    <t>demo1780943674478</t>
-  </si>
-  <si>
-    <t>demo1780943764355</t>
-  </si>
-  <si>
-    <t>demo1780943786860</t>
-  </si>
-  <si>
-    <t>demo1780943856986</t>
-  </si>
-  <si>
-    <t>demo1780943911225</t>
-  </si>
-  <si>
-    <t>demo1780943968400</t>
-  </si>
-  <si>
-    <t>demo1780943978392</t>
-  </si>
-  <si>
-    <t>demo1780944039395</t>
-  </si>
-  <si>
-    <t>demo1780944043093</t>
-  </si>
-  <si>
-    <t>demo1780944046193</t>
-  </si>
-  <si>
-    <t>demo1780944048780</t>
-  </si>
-  <si>
-    <t>demo1780944066716</t>
-  </si>
-  <si>
-    <t>demo1781103555232</t>
-  </si>
-  <si>
-    <t>demo1781103561528</t>
-  </si>
-  <si>
-    <t>demo1781103565477</t>
-  </si>
-  <si>
-    <t>demo1781103568609</t>
-  </si>
-  <si>
-    <t>demo1781103587277</t>
-  </si>
-  <si>
-    <t>demo1781116874993</t>
-  </si>
-  <si>
-    <t>demo1781116882382</t>
-  </si>
-  <si>
-    <t>demo1781116885969</t>
-  </si>
-  <si>
-    <t>demo1781116889006</t>
-  </si>
-  <si>
-    <t>demo1781116907345</t>
-  </si>
-  <si>
-    <t>demo1781117115396</t>
-  </si>
-  <si>
-    <t>demo1781117120364</t>
-  </si>
-  <si>
-    <t>demo1781117123565</t>
-  </si>
-  <si>
-    <t>demo1781117126277</t>
-  </si>
-  <si>
-    <t>demo1781117144676</t>
-  </si>
-  <si>
-    <t>demo1781117672003</t>
-  </si>
-  <si>
-    <t>demo1781117676866</t>
-  </si>
-  <si>
-    <t>demo1781117679826</t>
-  </si>
-  <si>
-    <t>demo1781117682413</t>
-  </si>
-  <si>
-    <t>demo1781117700858</t>
-  </si>
-  <si>
-    <t>demo1781122527209</t>
-  </si>
-  <si>
-    <t>demo1781122532477</t>
-  </si>
-  <si>
-    <t>demo1781122535396</t>
-  </si>
-  <si>
-    <t>demo1781122538091</t>
-  </si>
-  <si>
-    <t>demo1781122556310</t>
-  </si>
-  <si>
-    <t>demo1781157332726</t>
-  </si>
-  <si>
-    <t>demo1781157339018</t>
-  </si>
-  <si>
-    <t>demo1781157343224</t>
-  </si>
-  <si>
-    <t>demo1781157346185</t>
-  </si>
-  <si>
-    <t>demo1781157364695</t>
-  </si>
-  <si>
-    <t>demo1781174909134</t>
-  </si>
-  <si>
-    <t>demo1781174915227</t>
-  </si>
-  <si>
-    <t>demo1781174919209</t>
-  </si>
-  <si>
-    <t>demo1781174922070</t>
-  </si>
-  <si>
-    <t>demo1781174940365</t>
-  </si>
-  <si>
-    <t>demo1781174943441</t>
-  </si>
-  <si>
-    <t>demo1781174946886</t>
-  </si>
-  <si>
-    <t>demo1781175795099</t>
-  </si>
-  <si>
-    <t>demo1781175980780</t>
-  </si>
-  <si>
-    <t>demo1781176082479</t>
-  </si>
-  <si>
-    <t>demo1781176137273</t>
-  </si>
-  <si>
-    <t>demo1781176224165</t>
-  </si>
-  <si>
-    <t>demo1781209677848</t>
-  </si>
-  <si>
-    <t>demo1781209685958</t>
-  </si>
-  <si>
-    <t>demo1781209690355</t>
-  </si>
-  <si>
-    <t>demo1781209693462</t>
-  </si>
-  <si>
-    <t>demo1781209711982</t>
-  </si>
-  <si>
-    <t>demo1781209715752</t>
-  </si>
-  <si>
-    <t>demo1781209720116</t>
-  </si>
-  <si>
-    <t>demo1781210363962</t>
-  </si>
-  <si>
-    <t>demo1781210370839</t>
-  </si>
-  <si>
-    <t>demo1781210374868</t>
-  </si>
-  <si>
-    <t>demo1781210378045</t>
-  </si>
-  <si>
-    <t>demo1781210396495</t>
-  </si>
-  <si>
-    <t>demo1781210400063</t>
-  </si>
-  <si>
-    <t>demo1781210403618</t>
-  </si>
-  <si>
-    <t>demo1781210923757</t>
-  </si>
-  <si>
-    <t>demo1781210929768</t>
-  </si>
-  <si>
-    <t>demo1781210933423</t>
-  </si>
-  <si>
-    <t>demo1781210936552</t>
-  </si>
-  <si>
-    <t>demo1781210954790</t>
-  </si>
-  <si>
-    <t>demo1781210958217</t>
-  </si>
-  <si>
-    <t>demo1781210961611</t>
-  </si>
-  <si>
-    <t>demo1781289254147</t>
-  </si>
-  <si>
-    <t>demo1781289276796</t>
-  </si>
-  <si>
-    <t>demo1781289300167</t>
-  </si>
-  <si>
-    <t>demo1781289319680</t>
-  </si>
-  <si>
-    <t>demo1781289338201</t>
-  </si>
-  <si>
-    <t>demo1781289355268</t>
-  </si>
-  <si>
-    <t>demo1781289372362</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="10.0"/>
@@ -453,6 +178,10 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -659,7 +388,6 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -736,7 +464,6 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -746,13 +473,43 @@
       <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>124</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>17</v>
+      <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="1">
+        <v>141010.0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1.23456789E9</v>
+      </c>
+      <c r="G2" s="1">
+        <v>100.0</v>
       </c>
     </row>
   </sheetData>
@@ -765,23 +522,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -794,7 +542,26 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -807,10 +574,10 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed some issues with the excel file.
</commit_message>
<xml_diff>
--- a/ParabankAutomation/src/test/resources/TestData.xlsx
+++ b/ParabankAutomation/src/test/resources/TestData.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{4026F027-EBA4-4B2A-9E3E-DBEA0ED18281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Registration" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="BillPay" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="NegativeTestData" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="AccountData" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="LoginData" sheetId="5" r:id="rId9"/>
+    <sheet name="Registration" sheetId="1" r:id="rId1"/>
+    <sheet name="BillPay" sheetId="2" r:id="rId2"/>
+    <sheet name="NegativeTestData" sheetId="3" r:id="rId3"/>
+    <sheet name="AccountData" sheetId="4" r:id="rId4"/>
+    <sheet name="LoginData" sheetId="5" r:id="rId5"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:K13"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>First Name</t>
   </si>
@@ -115,22 +120,20 @@
   <si>
     <t>Type</t>
   </si>
-  <si>
-    <t>Hey</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -141,56 +144,43 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -380,17 +370,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -422,7 +415,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -439,10 +432,10 @@
         <v>14</v>
       </c>
       <c r="F2" s="1">
-        <v>10001.0</v>
+        <v>10001</v>
       </c>
       <c r="G2" s="1">
-        <v>9.87654321E9</v>
+        <v>9876543210</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>15</v>
@@ -455,18 +448,19 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -489,7 +483,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -503,28 +497,29 @@
         <v>28</v>
       </c>
       <c r="E2" s="1">
-        <v>141010.0</v>
+        <v>141010</v>
       </c>
       <c r="F2" s="1">
-        <v>1.23456789E9</v>
+        <v>1234567890</v>
       </c>
       <c r="G2" s="1">
-        <v>100.0</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -533,18 +528,19 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
@@ -553,18 +549,19 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -572,15 +569,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>